<commit_message>
docs: update SPPP and risk register for Iteration 2
</commit_message>
<xml_diff>
--- a/doc/CS673_SPPP_RiskManagement_team2.xlsx
+++ b/doc/CS673_SPPP_RiskManagement_team2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="98">
   <si>
     <t>This sheet provides some common risks in student projects. You should check if it applies to your group project. 
 You should also feel free to add other risks. Exemplary analysis is also added.</t>
@@ -75,7 +75,7 @@
     <t>Redefine the project scope if necessary, and assign the tasks to other team members.</t>
   </si>
   <si>
-    <t>Realized. Two members (Paul Probst, Victor Cadena) left the course before Iteration 1 work began; the team has been four members since 09/12/2026. Mitigation executed: roles reassigned (Design &amp; Implementation Leader added to Duc, Security Leader to Miles) and scope reduced in SPPP v2 (five features removed, two moved to a lower tier). Reopened with impact rescored from 4 to 5, since each further departure now costs a quarter of the team.</t>
+    <t>Realized. Two members (Paul Probst, Victor Cadena) left the course before Iteration 1 work began; the team has been four members since 09/12/2026. Mitigation executed: roles reassigned (Design &amp; Implementation Leader added to Duc, Security Leader to Miles) and scope reduced in SPPP v2 (five features removed, two moved to a lower tier). Reopened with impact rescored from 4 to 5, since each further departure now costs a quarter of the team. Iteration 2: no further departures; work was split into owned chunks across all four members.</t>
   </si>
   <si>
     <t>Open</t>
@@ -93,7 +93,7 @@
     <t>Track assignments and progress each iteration. Identify missed work early, redistribute tasks when necessary, and prioritize essential requirements over lower-priority work.</t>
   </si>
   <si>
-    <t>Iteration 1 work was split into owned workstreams with stated dependencies; all four were delivered and merged (PRs #8, #14, #16, #17).</t>
+    <t>Iteration 1 work was split into owned workstreams with stated dependencies; all four were delivered and merged (PRs #8, #14, #16, #17). Iteration 2: 11 chunks, each with a named owner, its dependencies, and a 'Done when' check, tracked in Discord and on the Jira sprint.</t>
   </si>
   <si>
     <t>Team member availability or uneven workload</t>
@@ -105,7 +105,7 @@
     <t>Divide essential functionality across the team while avoiding unnecessary single-person dependencies. Track work during each iteration, document implementation decisions, conduct code reviews, and redistribute tasks when workload or availability changes.</t>
   </si>
   <si>
-    <t>Iteration 1 used one owner per workstream. After the team reduction, implementation is shared by all four members rather than split between frontend and backend leads.</t>
+    <t>Iteration 1 used one owner per workstream. After the team reduction, implementation is shared by all four members rather than split between frontend and backend leads. Iteration 2: backend and frontend chunks were made independent (new response fields optional on the frontend), so a late chunk could not block anyone else's.</t>
   </si>
   <si>
     <t>Communication</t>
@@ -120,7 +120,7 @@
     <t>Assign ownership of tasks before development begins and track assignments using the team’s project-management system. Discuss current and upcoming work during team meetings.</t>
   </si>
   <si>
-    <t>The Iteration 1 plan assigned every file to exactly one workstream and routed shared files through a single owner; no duplicated work was identified.</t>
+    <t>The Iteration 1 plan assigned every file to exactly one workstream and routed shared files through a single owner; no duplicated work was identified. The Iteration 2 plan did the same, with an ownership rule for every shared file; no duplicated work.</t>
   </si>
   <si>
     <t>inconsistent work</t>
@@ -129,13 +129,10 @@
     <t>Independently developed frontend, backend, AI, and configuration components may make incompatible assumptions about interfaces, data structures, or behavior.</t>
   </si>
   <si>
-    <t>10/05/2026</t>
-  </si>
-  <si>
     <t>Define component interfaces and shared data structures before implementation. Communicate interface changes and integrate components regularly rather than waiting until the end of an iteration.</t>
   </si>
   <si>
-    <t>The API contract, database schema, and error format were published in the Iteration 1 plan before coding, and frontend and backend were built and integrated against them (PRs #14, #16, #17).</t>
+    <t>The API contract, database schema, and error format were published in the Iteration 1 plan before coding, and frontend and backend were built and integrated against them (PRs #14, #16, #17). Iteration 2: the API additions (due_counts, intervals) and each study component's props were agreed in the plan before coding.</t>
   </si>
   <si>
     <t xml:space="preserve">Requirements </t>
@@ -153,7 +150,7 @@
     <t>Define essential requirements as clear user stories with expected behavior. Review requirements with the team before implementation and clarify ambiguous requirements before development begins.</t>
   </si>
   <si>
-    <t>Requirements re-tiered and narrowed in SPPP v2; each remaining essential feature has a defined user story and scope.</t>
+    <t>Requirements re-tiered and narrowed in SPPP v2; each remaining essential feature has a defined user story and scope. Iteration 2: every chunk had a user story and Given/When/Then acceptance examples, and tests are named after them.</t>
   </si>
   <si>
     <t>scope creep</t>
@@ -168,7 +165,7 @@
     <t>Maintain the essential/desirable/optional classification. Require proposed additions to be evaluated against schedule and essential requirements. Defer new functionality to desirable or optional scope when it threatens essential work.</t>
   </si>
   <si>
-    <t>Scope reduced in SPPP v2 after the team shrank: five features removed and two moved to a lower tier. New work is evaluated against the remaining schedule before it is accepted.</t>
+    <t>Scope reduced in SPPP v2 after the team shrank: five features removed and two moved to a lower tier. New work is evaluated against the remaining schedule before it is accepted. Iteration 2: typed-answer mode was cut and AI generation moved to Iteration 3 to finish study mode; the plan lists what is out of scope.</t>
   </si>
   <si>
     <t>Management</t>
@@ -198,7 +195,7 @@
     <t>Estimate work by iteration, compare estimates with actual hours after each iteration, and revise later estimates and scope based on actual progress. Prioritize essential requirements when schedule pressure occurs.</t>
   </si>
   <si>
-    <t>Iteration 2 and 3 estimates revised for a four-person team in SPPP v2; actual hours are compared against estimates at the end of each iteration.</t>
+    <t>Iteration 2 and 3 estimates revised for a four-person team in SPPP v2; actual hours are compared against estimates at the end of each iteration. Realized in Iteration 2: AI deck generation, planned for this iteration, did not fit alongside study mode and was moved to Iteration 3. Mitigation executed: study mode prioritized and delivered complete, and Iteration 3 re-planned.</t>
   </si>
   <si>
     <t>Design and implementation</t>
@@ -216,7 +213,7 @@
     <t>Define the application’s major components, interfaces, and core card/deck/review data model early. Keep the card model generic rather than language-specific and review major design decisions with the team before implementation.</t>
   </si>
   <si>
-    <t>Schema, API contract, and error model were defined before implementation in Iteration 1. Schema changes are now versioned as database migrations and verified against the models in CI.</t>
+    <t>Schema, API contract, and error model were defined before implementation in Iteration 1. Schema changes are now versioned as database migrations and verified against the models in CI. Iteration 2 needed no schema changes; the scheduler is a pure module behind an interface frozen in Lab 3.</t>
   </si>
   <si>
     <t>LLM generates inaccurate or low-quality flashcards</t>
@@ -228,7 +225,7 @@
     <t>Use structured prompts and output validation. Allow users to review, edit, or delete generated cards. Test generation using representative prompts and subjects before release.</t>
   </si>
   <si>
-    <t>Not yet started; AI generation is scheduled for Iteration 2. Every generated card will be permanently flagged as AI-generated and remain editable, and model output is validated before it is saved.</t>
+    <t>Moved to Iteration 3 with AI generation. Planned controls unchanged: structured prompts, validation before saving, user review and editing, and a permanent AI-generated label.</t>
   </si>
   <si>
     <t xml:space="preserve">Testing </t>
@@ -243,7 +240,7 @@
     <t>Require unit testing of critical backend/SRS logic and integration testing of major workflows. Test essential features before desirable or optional features receive development priority.</t>
   </si>
   <si>
-    <t>Backend tests run against both SQLite and PostgreSQL on every pull request with a 90% minimum coverage gate; frontend lint and tests also run in CI.</t>
+    <t>Backend tests run against both SQLite and PostgreSQL on every pull request with a 90% minimum coverage gate; frontend lint and tests also run in CI. Iteration 2: the frontend moved to Vitest and React Testing Library, with component tests for every page and a 90% coverage gate (174 tests, 91.66%); the backend has 201 tests at 97.02%.</t>
   </si>
   <si>
     <t>Integration and deployment</t>
@@ -261,7 +258,7 @@
     <t>Establish the Docker environment and integration process early. Integrate frontend and backend incrementally and reserve time in each iteration for integration rather than postponing it until the end.</t>
   </si>
   <si>
-    <t>Docker environment in place, and CI builds the images and smoke-tests the full stack on every pull request. CD publishes images to GHCR; Render hosting hooks are not yet configured, so deploys are currently skipped.</t>
+    <t>Docker environment in place, and CI builds the images and smoke-tests the full stack on every pull request. CD publishes images to GHCR. Render deploy hooks are still not configured, so deploys are skipped and the demo runs on Docker Compose. Iteration 2: CI on develop failed when the image scan found OpenSSL vulnerabilities that a cached build layer had skipped patching; fixed in PR #44.</t>
   </si>
   <si>
     <t>Merge conflicts or incompatible code changes</t>
@@ -273,7 +270,7 @@
     <t>Use feature branches and pull requests, keep changes focused, merge frequently, review code before merging, and run automated tests or other integration checks before changes are accepted.</t>
   </si>
   <si>
-    <t>Feature branches and pull requests with a required review and required CI checks, enforced by a repository ruleset. One merge conflict (PR #16) was resolved before merge.</t>
+    <t>Feature branches and pull requests with a required review and required CI checks, enforced by a repository ruleset. One merge conflict (PR #16) was resolved before merge. Iteration 2: one owner per file, and the one planned overlap (B2 and B3 in api/decks.py) was confined to separate lines.</t>
   </si>
   <si>
     <t>LLM API availability, rate limits, or cost</t>
@@ -285,16 +282,47 @@
     <t>Isolate LLM access behind a service/API layer, handle API failures gracefully, limit unnecessary requests and deck-generation size, and avoid making non-AI application functionality dependent on API availability.</t>
   </si>
   <si>
-    <t>Not yet started; scheduled for Iteration 2. Controls specified in SPPP v2: LLM calls isolated server-side, capped prompt length and cards per request, a per-user daily limit, and every other feature works without the API.</t>
+    <t>Moved to Iteration 3. Planned controls unchanged: LLM calls isolated server-side, capped prompt length and cards per request, a per-user daily limit, and every other feature works without the API.</t>
+  </si>
+  <si>
+    <t>Third-party dependency changes and vulnerabilities</t>
+  </si>
+  <si>
+    <t>A new release of a dependency, or a newly published vulnerability, can break installs or fail CI with no change to our code.</t>
+  </si>
+  <si>
+    <t>Security Leader</t>
+  </si>
+  <si>
+    <t>10/13/2026</t>
+  </si>
+  <si>
+    <t>Pin dependencies that have broken us; scan both images with Trivy and run CodeQL on every pull request; keep Dependabot security alerts on; rebuild the OS-update layer of the frontend image on every build.</t>
+  </si>
+  <si>
+    <t>Realized twice in Iteration 2: SQLAlchemy 2.1 changed the default PostgreSQL driver and broke every connection (pinned to 2.0.54, PR #35); OpenSSL vulnerabilities failed the image scan on develop (PR #44).</t>
+  </si>
+  <si>
+    <t>Documents drift from the code</t>
+  </si>
+  <si>
+    <t>Design and test documents describe planned components rather than what was built, which misleads reviewers and teammates.</t>
+  </si>
+  <si>
+    <t>Update the SDD and STD from the code at the end of every iteration, in the release pull request, and label planned work as planned.</t>
+  </si>
+  <si>
+    <t>Realized: the Iteration 1 SDD described services, tables, and endpoints that were planned but not built. Corrected in the Iteration 2 SDD.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-    <numFmt numFmtId="165" formatCode="m/d"/>
+    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="166" formatCode="m/d"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -334,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -365,8 +393,11 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
@@ -374,10 +405,22 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -587,7 +630,7 @@
       <c r="J4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="8" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="5" t="s">
@@ -639,7 +682,7 @@
       <c r="J5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="8" t="s">
         <v>28</v>
       </c>
       <c r="L5" s="5" t="s">
@@ -693,7 +736,7 @@
       <c r="J6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="8" t="s">
         <v>33</v>
       </c>
       <c r="L6" s="5" t="s">
@@ -739,14 +782,14 @@
       <c r="H7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="10">
+        <v>46308.0</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="K7" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>38</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>19</v>
@@ -769,13 +812,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="D8" s="6">
         <v>3.0</v>
@@ -791,16 +834,16 @@
         <v>12</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I8" s="10">
+        <v>46308.0</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" s="5" t="s">
+      <c r="K8" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>19</v>
@@ -824,10 +867,10 @@
     <row r="9">
       <c r="A9" s="3"/>
       <c r="B9" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="6">
         <v>4.0</v>
@@ -843,16 +886,16 @@
         <v>4</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="J9" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>19</v>
@@ -875,13 +918,13 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="D10" s="6">
         <v>2.0</v>
@@ -897,16 +940,16 @@
         <v>16</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>22</v>
       </c>
       <c r="J10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>54</v>
-      </c>
-      <c r="K10" s="10" t="s">
-        <v>55</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>19</v>
@@ -930,10 +973,10 @@
     <row r="11">
       <c r="A11" s="3"/>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D11" s="6">
         <v>3.0</v>
@@ -949,16 +992,16 @@
         <v>9</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>59</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>19</v>
@@ -981,13 +1024,13 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="D12" s="6">
         <v>3.0</v>
@@ -1003,16 +1046,16 @@
         <v>9</v>
       </c>
       <c r="H12" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="10">
+        <v>46308.0</v>
+      </c>
+      <c r="J12" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="J12" s="5" t="s">
+      <c r="K12" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="K12" s="10" t="s">
-        <v>65</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>19</v>
@@ -1036,10 +1079,10 @@
     <row r="13">
       <c r="A13" s="2"/>
       <c r="B13" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="6">
         <v>4.0</v>
@@ -1055,16 +1098,16 @@
         <v>8</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
-      <c r="I13" s="6" t="s">
-        <v>36</v>
+      <c r="I13" s="10">
+        <v>46308.0</v>
       </c>
       <c r="J13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>69</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>19</v>
@@ -1087,16 +1130,16 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="6">
-        <v>3.0</v>
+      <c r="D14" s="11">
+        <v>2.0</v>
       </c>
       <c r="E14" s="6">
         <v>5.0</v>
@@ -1106,7 +1149,7 @@
       </c>
       <c r="G14" s="6">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>16</v>
@@ -1115,10 +1158,10 @@
         <v>22</v>
       </c>
       <c r="J14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>74</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>19</v>
@@ -1141,13 +1184,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="C15" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="D15" s="6">
         <v>3.0</v>
@@ -1163,16 +1206,16 @@
         <v>9</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>22</v>
       </c>
       <c r="J15" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="K15" s="10" t="s">
-        <v>80</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>19</v>
@@ -1196,10 +1239,10 @@
     <row r="16">
       <c r="A16" s="2"/>
       <c r="B16" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D16" s="6">
         <v>3.0</v>
@@ -1221,10 +1264,10 @@
         <v>22</v>
       </c>
       <c r="J16" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>84</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>19</v>
@@ -1248,10 +1291,10 @@
     <row r="17">
       <c r="A17" s="2"/>
       <c r="B17" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D17" s="6">
         <v>3.0</v>
@@ -1269,14 +1312,14 @@
       <c r="H17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>36</v>
+      <c r="I17" s="10">
+        <v>46308.0</v>
       </c>
       <c r="J17" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>87</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>88</v>
       </c>
       <c r="L17" s="5" t="s">
         <v>19</v>
@@ -1298,18 +1341,43 @@
       <c r="AA17" s="9"/>
     </row>
     <row r="18">
-      <c r="A18" s="12"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
+      <c r="A18" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="15">
+        <v>4.0</v>
+      </c>
+      <c r="E18" s="15">
+        <v>3.0</v>
+      </c>
+      <c r="F18" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="G18" s="16">
+        <f t="shared" ref="G18:G19" si="2">(6-D18)*(6-E18)*F18</f>
+        <v>6</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I18" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>19</v>
+      </c>
       <c r="M18" s="9"/>
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
@@ -1327,18 +1395,43 @@
       <c r="AA18" s="9"/>
     </row>
     <row r="19">
-      <c r="A19" s="9"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
+      <c r="A19" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="15">
+        <v>3.0</v>
+      </c>
+      <c r="E19" s="15">
+        <v>3.0</v>
+      </c>
+      <c r="F19" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="G19" s="16">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="J19" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L19" s="13" t="s">
+        <v>19</v>
+      </c>
       <c r="M19" s="9"/>
       <c r="N19" s="9"/>
       <c r="O19" s="9"/>
@@ -1359,15 +1452,15 @@
       <c r="A20" s="9"/>
       <c r="B20" s="4"/>
       <c r="C20" s="9"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
       <c r="H20" s="9"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="20"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9"/>
       <c r="O20" s="9"/>
@@ -1388,13 +1481,13 @@
       <c r="A21" s="9"/>
       <c r="B21" s="4"/>
       <c r="C21" s="9"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
       <c r="H21" s="9"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="15"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="20"/>
       <c r="K21" s="9"/>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
@@ -1417,15 +1510,15 @@
       <c r="A22" s="9"/>
       <c r="B22" s="4"/>
       <c r="C22" s="9"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
       <c r="H22" s="9"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
@@ -1446,16 +1539,16 @@
       <c r="A23" s="9"/>
       <c r="B23" s="4"/>
       <c r="C23" s="9"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
       <c r="H23" s="9"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
       <c r="P23" s="9"/>
@@ -1504,9 +1597,9 @@
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
@@ -1533,9 +1626,9 @@
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
@@ -1562,9 +1655,9 @@
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -1591,9 +1684,9 @@
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
@@ -1620,9 +1713,9 @@
       <c r="A29" s="9"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
@@ -1649,9 +1742,9 @@
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
       <c r="I30" s="9"/>
@@ -1678,7 +1771,7 @@
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
-      <c r="D31" s="13"/>
+      <c r="D31" s="16"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -1765,16 +1858,16 @@
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
       <c r="F34" s="9"/>
-      <c r="G34" s="13"/>
+      <c r="G34" s="16"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="20"/>
+      <c r="L34" s="20"/>
+      <c r="M34" s="20"/>
       <c r="N34" s="9"/>
       <c r="O34" s="9"/>
       <c r="P34" s="9"/>
@@ -1794,14 +1887,14 @@
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
       <c r="F35" s="9"/>
-      <c r="G35" s="13"/>
+      <c r="G35" s="16"/>
       <c r="H35" s="9"/>
       <c r="I35" s="9"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
@@ -1823,10 +1916,10 @@
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
       <c r="F36" s="9"/>
-      <c r="G36" s="13"/>
+      <c r="G36" s="16"/>
       <c r="H36" s="9"/>
       <c r="I36" s="9"/>
       <c r="J36" s="9"/>
@@ -1852,10 +1945,10 @@
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
       <c r="F37" s="9"/>
-      <c r="G37" s="13"/>
+      <c r="G37" s="16"/>
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
       <c r="J37" s="9"/>

</xml_diff>